<commit_message>
changed excel a bit added scatter graph to p8
</commit_message>
<xml_diff>
--- a/Excel_Handson2_Data_07.10.26.xlsx
+++ b/Excel_Handson2_Data_07.10.26.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ayaanjauhar/Desktop/IIM_Mumbai/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ayaanjauhar/Work/excel_python_project_2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D44E45F-0025-4F47-AA1F-579228CFD0B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08C6E9E8-3BA1-8840-B750-32E4C3D3F8BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="580" windowWidth="28800" windowHeight="18060" tabRatio="798" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="580" windowWidth="28800" windowHeight="18060" tabRatio="798" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Read me" sheetId="1" r:id="rId1"/>
@@ -26,13 +26,11 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'P6 Sales'!$F$5:$H$7</definedName>
-    <definedName name="_xlchart.v1.0" hidden="1">'P5 Shape'!$B$2:$B$121</definedName>
-    <definedName name="_xlchart.v1.1" hidden="1">'P5 Shape'!$E$2:$E$101</definedName>
-    <definedName name="_xlchart.v1.2" hidden="1">'P5 Shape'!$J$2:$J$6</definedName>
+    <definedName name="_xlchart.v1.0" hidden="1">'P5 Shape'!$E$2:$E$101</definedName>
+    <definedName name="_xlchart.v1.1" hidden="1">'P5 Shape'!$J$2:$J$6</definedName>
+    <definedName name="_xlchart.v1.2" hidden="1">'P5 Shape'!$B$2:$B$121</definedName>
     <definedName name="_xlchart.v1.3" hidden="1">'P7 Rents'!$B$1</definedName>
     <definedName name="_xlchart.v1.4" hidden="1">'P7 Rents'!$B$2:$B$41</definedName>
-    <definedName name="_xlchart.v1.5" hidden="1">'P7 Rents'!$B$1</definedName>
-    <definedName name="_xlchart.v1.6" hidden="1">'P7 Rents'!$B$2:$B$41</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -711,6 +709,7 @@
         <sz val="10"/>
         <color theme="1"/>
         <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
       </rPr>
       <t>PERCENTILE.INC</t>
     </r>
@@ -729,6 +728,7 @@
         <sz val="10"/>
         <color theme="1"/>
         <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
       </rPr>
       <t>.EXC</t>
     </r>
@@ -777,6 +777,7 @@
         <sz val="10"/>
         <color theme="1"/>
         <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
       </rPr>
       <t>KURT</t>
     </r>
@@ -1049,6 +1050,7 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial Unicode MS"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="8"/>
@@ -1169,17 +1171,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="11">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="10">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1341,12 +1333,854 @@
 </styleSheet>
 </file>
 
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-GB"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-GB"/>
+              <a:t>Hours</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-GB" baseline="0"/>
+              <a:t> vs Marks</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-GB"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="linear"/>
+            <c:dispRSqr val="0"/>
+            <c:dispEq val="0"/>
+          </c:trendline>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'P8 Students'!$B$2:$B$16</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="15"/>
+                <c:pt idx="0">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>13</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>15</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'P8 Students'!$D$2:$D$16</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="15"/>
+                <c:pt idx="0">
+                  <c:v>47</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>58</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>52</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>52</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>73</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>52</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>81</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>86</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>52</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>54</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>83</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>75</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>48</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>74</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>68</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-2E2F-8D42-80D9-1C984BA763C0}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="1373461504"/>
+        <c:axId val="1375057920"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="1373461504"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1375057920"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="1375057920"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1373461504"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-GB"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-GB"/>
+              <a:t>Social</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-GB" baseline="0"/>
+              <a:t> media vs Marks</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-GB"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="linear"/>
+            <c:dispRSqr val="0"/>
+            <c:dispEq val="0"/>
+          </c:trendline>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'P8 Students'!$C$2:$C$16</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="15"/>
+                <c:pt idx="0">
+                  <c:v>5.5</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>4.5999999999999996</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2.6</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2.6</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2.8</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>4.7</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>3.8</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>2.4</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>4.5</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>3.5</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>1.3</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>4.2</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>4.2</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>2.2999999999999998</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>2.6</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'P8 Students'!$D$2:$D$16</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="15"/>
+                <c:pt idx="0">
+                  <c:v>47</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>58</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>52</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>52</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>73</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>52</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>81</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>86</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>52</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>54</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>83</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>75</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>48</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>74</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>68</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-5637-9D40-8DF2-80928143DDEE}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="1647300992"/>
+        <c:axId val="1647302784"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="1647300992"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1647302784"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="1647302784"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1647300992"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/chartEx1.xml><?xml version="1.0" encoding="utf-8"?>
 <cx:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex">
   <cx:chartData>
     <cx:data id="0">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.0</cx:f>
+        <cx:f>_xlchart.v1.2</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>
@@ -1407,7 +2241,7 @@
   <cx:chartData>
     <cx:data id="0">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.1</cx:f>
+        <cx:f>_xlchart.v1.0</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>
@@ -1468,7 +2302,7 @@
   <cx:chartData>
     <cx:data id="0">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.2</cx:f>
+        <cx:f>_xlchart.v1.1</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>
@@ -1759,6 +2593,86 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors5.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors6.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="366">
   <cs:axisTitle>
@@ -3794,6 +4708,1038 @@
     <cs:fontRef idx="minor">
       <a:schemeClr val="tx1"/>
     </cs:fontRef>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style5.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style6.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
   </cs:wall>
 </cs:chartStyle>
 </file>
@@ -4120,14 +6066,91 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>57150</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>82550</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>1695450</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>158750</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E070B5F9-9F5B-F756-23A1-82CFB54B1C0E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>717550</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>107950</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>666750</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>184150</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Chart 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{60F630EC-1AE0-DF22-7CB7-4E50E2A030D9}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{F6C1BD7C-B2E7-5743-AF84-C05DAA8D6427}" name="Table3" displayName="Table3" ref="G1:J6" totalsRowShown="0" headerRowDxfId="10" dataDxfId="9">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{F6C1BD7C-B2E7-5743-AF84-C05DAA8D6427}" name="Table3" displayName="Table3" ref="G1:J6" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
   <autoFilter ref="G1:J6" xr:uid="{F6C1BD7C-B2E7-5743-AF84-C05DAA8D6427}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{C1C948A5-B475-B743-9870-2EFB273C73C5}" name="Metric" dataDxfId="8"/>
-    <tableColumn id="2" xr3:uid="{D386BE67-5D28-C242-9626-62D6B777AA15}" name="Daily Returns " dataDxfId="7"/>
-    <tableColumn id="3" xr3:uid="{B7B8604F-9A23-9840-B8CB-7D464F7D4D5A}" name="Heights " dataDxfId="6"/>
-    <tableColumn id="4" xr3:uid="{1D3A78DC-40FB-A849-90F3-26B2A0F44870}" name="Salaries " dataDxfId="5"/>
+    <tableColumn id="1" xr3:uid="{C1C948A5-B475-B743-9870-2EFB273C73C5}" name="Metric" dataDxfId="7"/>
+    <tableColumn id="2" xr3:uid="{D386BE67-5D28-C242-9626-62D6B777AA15}" name="Daily Returns " dataDxfId="6"/>
+    <tableColumn id="3" xr3:uid="{B7B8604F-9A23-9840-B8CB-7D464F7D4D5A}" name="Heights " dataDxfId="5"/>
+    <tableColumn id="4" xr3:uid="{1D3A78DC-40FB-A849-90F3-26B2A0F44870}" name="Salaries " dataDxfId="4"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -4920,6 +6943,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -9048,17 +11072,14 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="F16">
-    <cfRule type="cellIs" dxfId="4" priority="2" operator="greaterThan">
-      <formula>"3$D$1:$D$31"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="3" operator="greaterThan">
-      <formula>"3$D$1:$D$31"</formula>
+  <conditionalFormatting sqref="D1:D31">
+    <cfRule type="cellIs" dxfId="3" priority="1" operator="greaterThan">
+      <formula>3</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D1:D31">
-    <cfRule type="cellIs" dxfId="2" priority="1" operator="greaterThan">
-      <formula>3</formula>
+  <conditionalFormatting sqref="F16">
+    <cfRule type="cellIs" dxfId="2" priority="2" operator="greaterThan">
+      <formula>"3$D$1:$D$31"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -10055,14 +12076,14 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="E12">
-    <cfRule type="cellIs" dxfId="1" priority="2" operator="greaterThan">
-      <formula>"4$B$2:$B$41"</formula>
+  <conditionalFormatting sqref="B2:B41">
+    <cfRule type="cellIs" dxfId="1" priority="1" operator="greaterThan">
+      <formula>45.75</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B2:B41">
-    <cfRule type="cellIs" dxfId="0" priority="1" operator="greaterThan">
-      <formula>45.75</formula>
+  <conditionalFormatting sqref="E12">
+    <cfRule type="cellIs" dxfId="0" priority="2" operator="greaterThan">
+      <formula>"4$B$2:$B$41"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>